<commit_message>
updated excels, solved student leave issues and updated its workers, try to assign both sls in the same day to Priya
</commit_message>
<xml_diff>
--- a/Rota-LocalRun(Complete)/Files/Data Base.xlsx
+++ b/Rota-LocalRun(Complete)/Files/Data Base.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="67">
   <si>
     <t>Name</t>
   </si>
@@ -91,45 +91,51 @@
     <t>YES</t>
   </si>
   <si>
+    <t>Liliana</t>
+  </si>
+  <si>
     <t>Gabriel</t>
   </si>
   <si>
+    <t>Charlotte</t>
+  </si>
+  <si>
+    <t>Carla</t>
+  </si>
+  <si>
+    <t>Eji</t>
+  </si>
+  <si>
+    <t>Mark</t>
+  </si>
+  <si>
+    <t>Volodymyr</t>
+  </si>
+  <si>
+    <t>Catia</t>
+  </si>
+  <si>
+    <t>Raiyan</t>
+  </si>
+  <si>
+    <t>Ryan</t>
+  </si>
+  <si>
+    <t>Aysha</t>
+  </si>
+  <si>
+    <t>Jamie</t>
+  </si>
+  <si>
+    <t>Ann</t>
+  </si>
+  <si>
+    <t>Ellie</t>
+  </si>
+  <si>
     <t>Priya</t>
   </si>
   <si>
-    <t>Liliana</t>
-  </si>
-  <si>
-    <t>Charlotte</t>
-  </si>
-  <si>
-    <t>Eji</t>
-  </si>
-  <si>
-    <t>Mark</t>
-  </si>
-  <si>
-    <t>Volodymyr</t>
-  </si>
-  <si>
-    <t>Catia</t>
-  </si>
-  <si>
-    <t>Raiyan</t>
-  </si>
-  <si>
-    <t>Ryan</t>
-  </si>
-  <si>
-    <t>Aysha</t>
-  </si>
-  <si>
-    <t>Jamie</t>
-  </si>
-  <si>
-    <t>Ellie</t>
-  </si>
-  <si>
     <t>Sam</t>
   </si>
   <si>
@@ -166,7 +172,7 @@
     <t>Livy</t>
   </si>
   <si>
-    <t>Bema</t>
+    <t>Vani</t>
   </si>
   <si>
     <t>Anna</t>
@@ -188,6 +194,27 @@
   </si>
   <si>
     <t>Dr Elkady</t>
+  </si>
+  <si>
+    <t>Dr Khan</t>
+  </si>
+  <si>
+    <t>Dr Elmaghraby</t>
+  </si>
+  <si>
+    <t>Karen</t>
+  </si>
+  <si>
+    <t>Receptionist</t>
+  </si>
+  <si>
+    <t>Caroline</t>
+  </si>
+  <si>
+    <t>Heather</t>
+  </si>
+  <si>
+    <t>Femi</t>
   </si>
 </sst>
 </file>
@@ -558,7 +585,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:U33"/>
+  <dimension ref="A1:U41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -722,7 +749,7 @@
         <v>22</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>23</v>
@@ -737,28 +764,28 @@
         <v>24</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>23</v>
@@ -773,7 +800,7 @@
         <v>23</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="U3" s="2" t="s">
         <v>23</v>
@@ -802,19 +829,19 @@
         <v>24</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>23</v>
@@ -829,7 +856,7 @@
         <v>23</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="R4" s="2" t="s">
         <v>23</v>
@@ -906,7 +933,7 @@
         <v>24</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
@@ -968,10 +995,10 @@
         <v>23</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
@@ -1340,7 +1367,7 @@
         <v>24</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O12" s="2" t="s">
         <v>24</v>
@@ -1405,7 +1432,7 @@
         <v>23</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O13" s="2" t="s">
         <v>24</v>
@@ -1529,7 +1556,7 @@
         <v>24</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M15" s="2" t="s">
         <v>23</v>
@@ -1544,7 +1571,7 @@
         <v>23</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="R15" s="2" t="s">
         <v>23</v>
@@ -1603,7 +1630,7 @@
         <v>23</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>23</v>
@@ -1632,34 +1659,34 @@
         <v>22</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M17" s="2" t="s">
         <v>23</v>
@@ -1667,17 +1694,27 @@
       <c r="N17" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
+      <c r="O17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="Q17" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="R17" s="2"/>
+        <v>24</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="S17" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
+      <c r="T17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U17" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="2" t="s">
@@ -1686,36 +1723,70 @@
       <c r="B18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
+      <c r="C18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="Q18" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="R18" s="2"/>
+      <c r="R18" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="S18" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T18" s="2"/>
-      <c r="U18" s="2"/>
+      <c r="T18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U18" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>24</v>
@@ -1727,7 +1798,7 @@
         <v>24</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>23</v>
@@ -1757,7 +1828,7 @@
         <v>24</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>23</v>
@@ -1777,43 +1848,43 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>24</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N20" s="2" t="s">
         <v>23</v>
@@ -1822,7 +1893,7 @@
         <v>23</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>23</v>
@@ -1842,11 +1913,11 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="C21" s="2" t="s">
         <v>24</v>
       </c>
@@ -1860,31 +1931,31 @@
         <v>24</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N21" s="2" t="s">
         <v>23</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>24</v>
@@ -1910,16 +1981,16 @@
         <v>45</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>24</v>
@@ -1975,13 +2046,13 @@
         <v>46</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>24</v>
@@ -1990,13 +2061,13 @@
         <v>24</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>24</v>
@@ -2040,19 +2111,19 @@
         <v>47</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>24</v>
@@ -2073,7 +2144,7 @@
         <v>23</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N24" s="2" t="s">
         <v>23</v>
@@ -2082,7 +2153,7 @@
         <v>23</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q24" s="2" t="s">
         <v>23</v>
@@ -2091,7 +2162,7 @@
         <v>23</v>
       </c>
       <c r="S24" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="T24" s="2" t="s">
         <v>23</v>
@@ -2105,19 +2176,19 @@
         <v>48</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>24</v>
@@ -2138,7 +2209,7 @@
         <v>23</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N25" s="2" t="s">
         <v>23</v>
@@ -2170,7 +2241,7 @@
         <v>49</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>23</v>
@@ -2197,7 +2268,7 @@
         <v>24</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>23</v>
@@ -2221,7 +2292,7 @@
         <v>23</v>
       </c>
       <c r="S26" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="T26" s="2" t="s">
         <v>23</v>
@@ -2235,7 +2306,7 @@
         <v>50</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>23</v>
@@ -2244,19 +2315,19 @@
         <v>23</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>23</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>24</v>
@@ -2300,38 +2371,72 @@
         <v>51</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2"/>
-      <c r="P28" s="2"/>
+        <v>44</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P28" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="Q28" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="R28" s="2"/>
+      <c r="R28" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="S28" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T28" s="2"/>
-      <c r="U28" s="2"/>
+      <c r="T28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U28" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>23</v>
@@ -2340,31 +2445,31 @@
         <v>23</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N29" s="2" t="s">
         <v>23</v>
@@ -2372,21 +2477,31 @@
       <c r="O29" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="P29" s="2"/>
-      <c r="Q29" s="2"/>
-      <c r="R29" s="2"/>
-      <c r="S29" s="2"/>
+      <c r="P29" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q29" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R29" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S29" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="T29" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="U29" s="2"/>
+      <c r="U29" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>23</v>
@@ -2401,25 +2516,25 @@
         <v>23</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>24</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N30" s="2" t="s">
         <v>23</v>
@@ -2427,22 +2542,32 @@
       <c r="O30" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="2"/>
-      <c r="S30" s="2"/>
+      <c r="P30" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q30" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R30" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S30" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="T30" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="U30" s="2"/>
+      <c r="U30" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="C31" s="2" t="s">
         <v>23</v>
       </c>
@@ -2462,7 +2587,7 @@
         <v>23</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>23</v>
@@ -2482,21 +2607,31 @@
       <c r="O31" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="P31" s="2"/>
-      <c r="Q31" s="2"/>
-      <c r="R31" s="2"/>
-      <c r="S31" s="2"/>
+      <c r="P31" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q31" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R31" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S31" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="T31" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="U31" s="2"/>
+      <c r="U31" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="2" t="s">
         <v>56</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>23</v>
@@ -2520,16 +2655,16 @@
         <v>23</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L32" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N32" s="2" t="s">
         <v>23</v>
@@ -2537,21 +2672,31 @@
       <c r="O32" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="P32" s="2"/>
-      <c r="Q32" s="2"/>
-      <c r="R32" s="2"/>
-      <c r="S32" s="2"/>
+      <c r="P32" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q32" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R32" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S32" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="T32" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="U32" s="2"/>
+      <c r="U32" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>23</v>
@@ -2572,7 +2717,7 @@
         <v>23</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J33" s="2" t="s">
         <v>23</v>
@@ -2584,7 +2729,7 @@
         <v>23</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N33" s="2" t="s">
         <v>23</v>
@@ -2608,6 +2753,450 @@
         <v>23</v>
       </c>
       <c r="U33" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+      <c r="A34" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T34" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U34" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+      <c r="A35" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U35" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+      <c r="A36" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="2"/>
+      <c r="R36" s="2"/>
+      <c r="S36" s="2"/>
+      <c r="T36" s="2"/>
+      <c r="U36" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+      <c r="A37" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="P37" s="2"/>
+      <c r="Q37" s="2"/>
+      <c r="R37" s="2"/>
+      <c r="S37" s="2"/>
+      <c r="T37" s="2"/>
+      <c r="U37" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+      <c r="A38" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S38" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U38" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+      <c r="A39" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S39" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T39" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U39" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
+      <c r="A40" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S40" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U40" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+      <c r="A41" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S41" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U41" s="2" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>